<commit_message>
Updated attribute collection list 2026.04.01
- Addition of reduction factor for intermittent heating (F_red_htr1 and 4). Responsible for contribution towards reduction in heat demand due to differences in continuous and intermittent heating.
</commit_message>
<xml_diff>
--- a/attribute-spec/Attribute_requirement_collection.xlsx
+++ b/attribute-spec/Attribute_requirement_collection.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29575CA6-6941-45A7-9025-A0074793B599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="805" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="805" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="3D-BAG" sheetId="1" r:id="rId1"/>
@@ -747,7 +747,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -776,20 +776,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
@@ -802,7 +793,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Explanatory Text" xfId="1" builtinId="53"/>
@@ -1084,17 +1078,17 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
@@ -1250,7 +1244,7 @@
       <c r="H8" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="I8" s="17" t="s">
+      <c r="I8" s="14" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1279,7 +1273,7 @@
       <c r="H9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="I9" s="17" t="s">
+      <c r="I9" s="14" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1308,7 +1302,7 @@
       <c r="H10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="I10" s="17" t="s">
+      <c r="I10" s="14" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1337,7 +1331,7 @@
       <c r="H11" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="I11" s="17" t="s">
+      <c r="I11" s="14" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1366,36 +1360,36 @@
       <c r="H12" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="I12" s="17" t="s">
+      <c r="I12" s="14" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="13" spans="1:9" s="20" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="18" t="s">
+    <row r="13" spans="1:9" s="17" customFormat="1" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="F13" s="18" t="s">
+      <c r="D13" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G13" s="18" t="s">
+      <c r="G13" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="18" t="s">
+      <c r="H13" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="I13" s="19" t="s">
+      <c r="I13" s="16" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1456,17 +1450,17 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
@@ -1994,7 +1988,7 @@
       <c r="A25" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="10" t="s">
         <v>136</v>
       </c>
       <c r="C25" s="1" t="s">
@@ -2467,7 +2461,7 @@
       <c r="A45" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B45" s="11" t="s">
+      <c r="B45" s="10" t="s">
         <v>137</v>
       </c>
       <c r="C45" s="1" t="s">
@@ -2485,7 +2479,7 @@
       <c r="G45" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="I45" s="13" t="s">
+      <c r="I45" s="1" t="s">
         <v>109</v>
       </c>
     </row>
@@ -2545,7 +2539,7 @@
       <c r="A48" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B48" s="11" t="s">
+      <c r="B48" s="10" t="s">
         <v>141</v>
       </c>
       <c r="C48" s="1" t="s">
@@ -2563,7 +2557,7 @@
       <c r="G48" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="I48" s="13" t="s">
+      <c r="I48" s="1" t="s">
         <v>142</v>
       </c>
     </row>
@@ -2571,7 +2565,7 @@
       <c r="A49" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B49" s="11" t="s">
+      <c r="B49" s="10" t="s">
         <v>143</v>
       </c>
       <c r="C49" s="1" t="s">
@@ -2589,7 +2583,7 @@
       <c r="G49" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="I49" s="15" t="s">
+      <c r="I49" s="8" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2597,7 +2591,7 @@
       <c r="A50" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B50" s="11" t="s">
+      <c r="B50" s="10" t="s">
         <v>144</v>
       </c>
       <c r="C50" s="1" t="s">
@@ -2615,7 +2609,7 @@
       <c r="G50" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="I50" s="15" t="s">
+      <c r="I50" s="8" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2623,7 +2617,7 @@
       <c r="A51" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B51" s="14" t="s">
+      <c r="B51" s="12" t="s">
         <v>145</v>
       </c>
       <c r="C51" s="1" t="s">
@@ -2641,7 +2635,7 @@
       <c r="G51" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="I51" s="15" t="s">
+      <c r="I51" s="8" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2649,7 +2643,7 @@
       <c r="A52" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B52" s="11" t="s">
+      <c r="B52" s="10" t="s">
         <v>146</v>
       </c>
       <c r="C52" s="1" t="s">
@@ -2667,7 +2661,7 @@
       <c r="G52" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="I52" s="15" t="s">
+      <c r="I52" s="8" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2675,7 +2669,7 @@
       <c r="A53" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B53" s="11" t="s">
+      <c r="B53" s="10" t="s">
         <v>148</v>
       </c>
       <c r="C53" s="1" t="s">
@@ -2693,7 +2687,7 @@
       <c r="G53" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="I53" s="13" t="s">
+      <c r="I53" s="1" t="s">
         <v>147</v>
       </c>
     </row>
@@ -2753,17 +2747,17 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
@@ -2795,10 +2789,10 @@
       <c r="F4" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="13" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2819,10 +2813,10 @@
       <c r="F5" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="I5" s="13" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2843,10 +2837,10 @@
       <c r="F6" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="16" t="s">
+      <c r="I6" s="13" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2857,19 +2851,19 @@
       <c r="C7" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D7" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="11" t="s">
+      <c r="D7" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>24</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="I7" s="11" t="s">
         <v>132</v>
       </c>
     </row>
@@ -2880,19 +2874,19 @@
       <c r="C8" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D8" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E8" s="11" t="s">
+      <c r="D8" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="10" t="s">
         <v>24</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="15" t="s">
+      <c r="I8" s="8" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2903,19 +2897,19 @@
       <c r="C9" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D9" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" s="11" t="s">
+      <c r="D9" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="10" t="s">
         <v>14</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I9" s="12" t="s">
+      <c r="I9" s="11" t="s">
         <v>135</v>
       </c>
     </row>
@@ -2926,19 +2920,19 @@
       <c r="C10" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D10" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="11" t="s">
+      <c r="D10" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>14</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="11" t="s">
         <v>135</v>
       </c>
     </row>
@@ -2949,19 +2943,19 @@
       <c r="C11" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D11" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E11" s="11" t="s">
+      <c r="D11" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="10" t="s">
         <v>24</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I11" s="12" t="s">
+      <c r="I11" s="11" t="s">
         <v>102</v>
       </c>
     </row>
@@ -2972,19 +2966,19 @@
       <c r="C12" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D12" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E12" s="11" t="s">
+      <c r="D12" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="10" t="s">
         <v>24</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="G12" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I12" s="12" t="s">
+      <c r="I12" s="11" t="s">
         <v>102</v>
       </c>
     </row>
@@ -2995,19 +2989,19 @@
       <c r="C13" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D13" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="11" t="s">
+      <c r="D13" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="10" t="s">
         <v>24</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="G13" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="12" t="s">
+      <c r="I13" s="11" t="s">
         <v>102</v>
       </c>
     </row>
@@ -3018,19 +3012,19 @@
       <c r="C14" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D14" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E14" s="11" t="s">
+      <c r="D14" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="10" t="s">
         <v>24</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="G14" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I14" s="15" t="s">
+      <c r="I14" s="8" t="s">
         <v>104</v>
       </c>
     </row>
@@ -3041,19 +3035,19 @@
       <c r="C15" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D15" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E15" s="11" t="s">
+      <c r="D15" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>24</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="G15" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I15" s="15" t="s">
+      <c r="I15" s="8" t="s">
         <v>104</v>
       </c>
     </row>
@@ -3064,19 +3058,19 @@
       <c r="C16" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D16" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="E16" s="11" t="s">
+      <c r="D16" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" s="10" t="s">
         <v>24</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="I16" s="15" t="s">
+      <c r="I16" s="8" t="s">
         <v>104</v>
       </c>
     </row>
@@ -3135,17 +3129,17 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -3167,7 +3161,7 @@
       <c r="G3" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="I3" s="13" t="s">
         <v>104</v>
       </c>
     </row>
@@ -3191,7 +3185,7 @@
       <c r="G4" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="13" t="s">
         <v>104</v>
       </c>
     </row>
@@ -3215,7 +3209,7 @@
       <c r="G5" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="I5" s="13" t="s">
         <v>104</v>
       </c>
     </row>
@@ -3239,7 +3233,7 @@
       <c r="G6" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="I6" s="16" t="s">
+      <c r="I6" s="13" t="s">
         <v>104</v>
       </c>
     </row>

</xml_diff>